<commit_message>
fix: paleta neutra no xlsx de copies (remove cor de marca de terceiros)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copy/COPYS_FASE1_AWARENESS.xlsx
+++ b/copy/COPYS_FASE1_AWARENESS.xlsx
@@ -49,7 +49,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000A6B63"/>
+      <color rgb="001F4E79"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -62,7 +62,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000A6B63"/>
+        <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>

</xml_diff>